<commit_message>
mistral testset getest met andere parameters. Goede verbetering
</commit_message>
<xml_diff>
--- a/evaluation/test_vragen_mistral.xlsx
+++ b/evaluation/test_vragen_mistral.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thoma\ACS\Internship\Realisatie\Stage\evaluation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6DBBF029-502E-46CB-AEF0-300784321A66}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F3D24B3-72F3-42DC-B477-5FE4ACB718EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="101">
   <si>
     <t>ID</t>
   </si>
@@ -283,6 +283,51 @@
   </si>
   <si>
     <t>Goed antwoord, bevat wel link in antwoord dus prompt opvolgen kan beter</t>
+  </si>
+  <si>
+    <t>Met chunk size 512 en top k 40 en overlap van 100 -&gt; 200</t>
+  </si>
+  <si>
+    <t>zelfde resultaat</t>
+  </si>
+  <si>
+    <t>Geeft ook Proctorio maar geeft meer uitleg dat eigenlijk niet nodig is</t>
+  </si>
+  <si>
+    <t>score van 0 -&gt; 1,5. chunk met stappen si er wel alleen wordt stap 4 genegeerd door bepertke chunk size en niet in andere chunk meegegeven</t>
+  </si>
+  <si>
+    <t>Zelfde probleem</t>
+  </si>
+  <si>
+    <t>Score van 0 -&gt; 2: chunk wordt gevonden met info en antwoord is goed</t>
+  </si>
+  <si>
+    <t>Zelfde</t>
+  </si>
+  <si>
+    <t>score van 0-&gt;2 perfect antwoord + retrieval</t>
+  </si>
+  <si>
+    <t>score van 2 -&gt; 1 , ideale chunk wordt niet gevonden maar er zit wel i juiste informatie in andere  chunks</t>
+  </si>
+  <si>
+    <t>zelfde</t>
+  </si>
+  <si>
+    <t>Net beter antwoord wat betreft stappen, maar meer overbodige stappen die niet nodig zijn, wel zelfde score</t>
+  </si>
+  <si>
+    <t>score van 0 -&gt; 2: correcte chunk gevonden enkel +- 7minuten niet vermeld maar wel de stap waarbij dit hoorde</t>
+  </si>
+  <si>
+    <t>score van 1 -&gt; 2 : vollediger en vermeld 50</t>
+  </si>
+  <si>
+    <t>zelde</t>
+  </si>
+  <si>
+    <t>zelfde, focust enkel op proctorio</t>
   </si>
 </sst>
 </file>
@@ -612,7 +657,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F23"/>
+  <dimension ref="A1:G24"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.6640625" customWidth="1"/>
@@ -621,9 +666,10 @@
     <col min="4" max="4" width="26" customWidth="1"/>
     <col min="5" max="5" width="5" customWidth="1"/>
     <col min="6" max="6" width="95.6640625" customWidth="1"/>
+    <col min="7" max="7" width="47.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -642,8 +688,11 @@
       <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="G1" s="1" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
@@ -662,8 +711,11 @@
       <c r="F2" s="2" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="G2" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2</v>
       </c>
@@ -682,8 +734,11 @@
       <c r="F3" s="2" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="G3" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>3</v>
       </c>
@@ -702,8 +757,11 @@
       <c r="F4" s="2" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="G4" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>4</v>
       </c>
@@ -722,8 +780,11 @@
       <c r="F5" s="2" t="s">
         <v>70</v>
       </c>
-    </row>
-    <row r="6" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="G5" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>5</v>
       </c>
@@ -742,8 +803,11 @@
       <c r="F6" s="2" t="s">
         <v>71</v>
       </c>
-    </row>
-    <row r="7" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="G6" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>6</v>
       </c>
@@ -762,8 +826,11 @@
       <c r="F7" s="2" t="s">
         <v>72</v>
       </c>
-    </row>
-    <row r="8" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="G7" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>7</v>
       </c>
@@ -782,8 +849,11 @@
       <c r="F8" s="2" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="9" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="G8" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>8</v>
       </c>
@@ -802,8 +872,11 @@
       <c r="F9" s="2" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="10" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="G9" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>9</v>
       </c>
@@ -822,8 +895,11 @@
       <c r="F10" s="2" t="s">
         <v>75</v>
       </c>
-    </row>
-    <row r="11" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="G10" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>10</v>
       </c>
@@ -842,8 +918,11 @@
       <c r="F11" s="2" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G11" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>11</v>
       </c>
@@ -862,8 +941,11 @@
       <c r="F12" s="2" t="s">
         <v>76</v>
       </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G12" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>12</v>
       </c>
@@ -882,8 +964,11 @@
       <c r="F13" s="2" t="s">
         <v>77</v>
       </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G13" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>13</v>
       </c>
@@ -902,8 +987,11 @@
       <c r="F14" s="2" t="s">
         <v>78</v>
       </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G14" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>14</v>
       </c>
@@ -922,8 +1010,11 @@
       <c r="F15" s="2" t="s">
         <v>79</v>
       </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G15" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>15</v>
       </c>
@@ -942,8 +1033,11 @@
       <c r="F16" s="2" t="s">
         <v>80</v>
       </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G16" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>16</v>
       </c>
@@ -962,8 +1056,11 @@
       <c r="F17" s="2" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="18" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="G17" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>17</v>
       </c>
@@ -982,8 +1079,11 @@
       <c r="F18" s="2" t="s">
         <v>81</v>
       </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G18" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>18</v>
       </c>
@@ -1002,8 +1102,11 @@
       <c r="F19" s="2" t="s">
         <v>82</v>
       </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G19" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>19</v>
       </c>
@@ -1022,8 +1125,11 @@
       <c r="F20" s="2" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G20" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>20</v>
       </c>
@@ -1042,8 +1148,11 @@
       <c r="F21" s="2" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="22" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="G21" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>21</v>
       </c>
@@ -1062,8 +1171,11 @@
       <c r="F22" s="2" t="s">
         <v>84</v>
       </c>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G22" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>22</v>
       </c>
@@ -1082,8 +1194,20 @@
       <c r="F23" s="2" t="s">
         <v>85</v>
       </c>
+      <c r="G23" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="E24">
+        <v>31</v>
+      </c>
+      <c r="G24">
+        <v>38.5</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
lichte aanpassing in excel file. Prompting gaf niet veel goeds nu dus kom hier later op terug
</commit_message>
<xml_diff>
--- a/evaluation/test_vragen_mistral.xlsx
+++ b/evaluation/test_vragen_mistral.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thoma\ACS\Internship\Realisatie\Stage\evaluation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F3D24B3-72F3-42DC-B477-5FE4ACB718EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB5D8096-EE60-45D2-962E-0DEF5EDD5F7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="87">
   <si>
     <t>ID</t>
   </si>
@@ -42,9 +42,6 @@
     <t>Score (0 =fout, 1=half, 2=juist)</t>
   </si>
   <si>
-    <t>Probleem</t>
-  </si>
-  <si>
     <t>Wat is het verschil tussen Schoolyear en Proctorio?</t>
   </si>
   <si>
@@ -129,9 +126,6 @@
     <t>nee- wordt overgenomen van Canvas</t>
   </si>
   <si>
-    <t>Relevante chunk aanwezig in retrieval, maar verwijderd door reranker omdat het antwoord impliciet geformuleerd is en niet exact overeenkomt met de vraag.</t>
-  </si>
-  <si>
     <t>Hoe kan ik video’s uploaden en gebruiken in Kaltura voor mijn cursus?</t>
   </si>
   <si>
@@ -174,9 +168,6 @@
     <t>focus op één thema - max ±7 minuten - duidelijke structuur - headset gebruiken - eenvoudige opzet</t>
   </si>
   <si>
-    <t>query te algemeen, relevante chunk niet opgehaald</t>
-  </si>
-  <si>
     <t>Heb ik nog toegang tot Canvas na mijn afstuderen?</t>
   </si>
   <si>
@@ -231,18 +222,9 @@
     <t>Antwoord inhoudelijks correct en gebaseerd op juiste context. Retrieval en reranking goed. Anwrood bevat bijkomende informatie die overbodig kan beschouwd worden dus model kiest voor volledigheid over beknoptheid.</t>
   </si>
   <si>
-    <t>Correct en beknopt antwoord met juiste bronselectie. Geen problemen in retrieval of reranking. Antwoord is direct en passend bij het vraagtype.</t>
-  </si>
-  <si>
-    <t>Fout antwoord door ontbrekende relevante context. De specifieke stappen voor activatie worden niet opgehaald, waardoor het model een incorrect stappenplan genereert. Probleem ligt bij retrieval (niet bij model of reranker).</t>
-  </si>
-  <si>
     <t>Antwoord is gedeeltelijk correct maar onvolledig. De context bevat niet de volledige checklist van vereisten voor studenten, waardoor het model slechts een deel van de informatie geeft en aanvullende elementen invult die niet expliciet in de context staan. Probleem ligt bij retrieval: de sectie met “Wat moeten studenten hebben en weten?” wordt niet opgehaald.</t>
   </si>
   <si>
-    <t>Geen antwoord door ontbreken van relevante chunks na reranking. De specifieke informatie (waarschuwing rond toegangscode) wordt niet opgehaald of scoort te laag, waardoor de pipeline onterecht overschakelt naar de intake-flow. Wel geen intent irrelevant maar support dus intake start</t>
-  </si>
-  <si>
     <t>Fout antwoord door verkeerde interpretatie van context. De vermelding van “kennisclips” wordt foutief geïnterpreteerd als functionaliteit van Proctorio.</t>
   </si>
   <si>
@@ -255,24 +237,15 @@
     <t>Correct en volledig antwoord met duidelijke stappenstructuur. Bevat beperkte extra informatie die niet strikt noodzakelijk is maar wel binnen scope vraag, maar volgt de instructies correct.</t>
   </si>
   <si>
-    <t>Alle nodige info aanwezig in context. Goed antwoord maar lichte overbodig informatie</t>
-  </si>
-  <si>
     <t>Juiste informatie gegeven, lichte overbodige info erbij maar acceptabel</t>
   </si>
   <si>
     <t>Goed antwoord en goede retrieval</t>
   </si>
   <si>
-    <t>Kort en bondig antwoord met 3 volledige stappen</t>
-  </si>
-  <si>
     <t>Kort en bondig antwoord, maar bevat alles</t>
   </si>
   <si>
-    <t>Antwoord is gedeeltelijk correct maar mist cruciale nuance: gebruikers behouden nog tijdelijk toegang (50 dagen) na afstuderen.</t>
-  </si>
-  <si>
     <t>Bevat alle info en is correct</t>
   </si>
   <si>
@@ -285,49 +258,34 @@
     <t>Goed antwoord, bevat wel link in antwoord dus prompt opvolgen kan beter</t>
   </si>
   <si>
-    <t>Met chunk size 512 en top k 40 en overlap van 100 -&gt; 200</t>
-  </si>
-  <si>
-    <t>zelfde resultaat</t>
-  </si>
-  <si>
-    <t>Geeft ook Proctorio maar geeft meer uitleg dat eigenlijk niet nodig is</t>
-  </si>
-  <si>
-    <t>score van 0 -&gt; 1,5. chunk met stappen si er wel alleen wordt stap 4 genegeerd door bepertke chunk size en niet in andere chunk meegegeven</t>
-  </si>
-  <si>
-    <t>Zelfde probleem</t>
-  </si>
-  <si>
-    <t>Score van 0 -&gt; 2: chunk wordt gevonden met info en antwoord is goed</t>
-  </si>
-  <si>
-    <t>Zelfde</t>
-  </si>
-  <si>
-    <t>score van 0-&gt;2 perfect antwoord + retrieval</t>
-  </si>
-  <si>
-    <t>score van 2 -&gt; 1 , ideale chunk wordt niet gevonden maar er zit wel i juiste informatie in andere  chunks</t>
-  </si>
-  <si>
-    <t>zelfde</t>
-  </si>
-  <si>
-    <t>Net beter antwoord wat betreft stappen, maar meer overbodige stappen die niet nodig zijn, wel zelfde score</t>
-  </si>
-  <si>
-    <t>score van 0 -&gt; 2: correcte chunk gevonden enkel +- 7minuten niet vermeld maar wel de stap waarbij dit hoorde</t>
-  </si>
-  <si>
-    <t>score van 1 -&gt; 2 : vollediger en vermeld 50</t>
-  </si>
-  <si>
-    <t>zelde</t>
-  </si>
-  <si>
-    <t>zelfde, focust enkel op proctorio</t>
+    <t>Correct en beknopt antwoord met juiste bronselectie. Geen problemen in retrieval of reranking. Antwoord is direct en passend bij het vraagtype. Geeft misschien wat te veel info</t>
+  </si>
+  <si>
+    <t>Juiste informatie maar mist 1 stap omdat die uit chunk valt en niet in andere chunk aanwezig is bij top k</t>
+  </si>
+  <si>
+    <t>Chunk wordt gevonden en antwoord is goed</t>
+  </si>
+  <si>
+    <t>Analyse</t>
+  </si>
+  <si>
+    <t>Heel goed antwoord + retrieval</t>
+  </si>
+  <si>
+    <t>Retrieval deels aanwezig, dus antwoord half correct</t>
+  </si>
+  <si>
+    <t>Goed antwoord, maar iets te veel overbodige info</t>
+  </si>
+  <si>
+    <t>Alles goed, enkel +- 7minuten wordt niet specifiek vermeld maar wel stap die deze info bevatte</t>
+  </si>
+  <si>
+    <t>Goed antwoord + retrieval</t>
+  </si>
+  <si>
+    <t>38,5/44</t>
   </si>
 </sst>
 </file>
@@ -664,7 +622,7 @@
     <col min="2" max="2" width="56.44140625" customWidth="1"/>
     <col min="3" max="3" width="18.88671875" customWidth="1"/>
     <col min="4" max="4" width="26" customWidth="1"/>
-    <col min="5" max="5" width="5" customWidth="1"/>
+    <col min="5" max="5" width="7.33203125" customWidth="1"/>
     <col min="6" max="6" width="95.6640625" customWidth="1"/>
     <col min="7" max="7" width="47.5546875" customWidth="1"/>
   </cols>
@@ -686,33 +644,28 @@
         <v>4</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>86</v>
-      </c>
+        <v>80</v>
+      </c>
+      <c r="G1" s="1"/>
     </row>
     <row r="2" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" t="s">
         <v>6</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>7</v>
       </c>
-      <c r="D2" t="s">
-        <v>8</v>
-      </c>
       <c r="E2">
         <v>2</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="G2" t="s">
-        <v>87</v>
+        <v>64</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -720,45 +673,39 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C3" t="s">
         <v>9</v>
       </c>
-      <c r="C3" t="s">
+      <c r="D3" t="s">
         <v>10</v>
       </c>
-      <c r="D3" t="s">
-        <v>11</v>
-      </c>
       <c r="E3">
         <v>2</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="G3" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>3</v>
       </c>
       <c r="B4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" t="s">
         <v>12</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
         <v>13</v>
       </c>
-      <c r="D4" t="s">
-        <v>14</v>
-      </c>
       <c r="E4">
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="G4" t="s">
-        <v>89</v>
+        <v>78</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
@@ -766,45 +713,39 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
+        <v>14</v>
+      </c>
+      <c r="C5" t="s">
         <v>15</v>
       </c>
-      <c r="C5" t="s">
+      <c r="D5" t="s">
         <v>16</v>
-      </c>
-      <c r="D5" t="s">
-        <v>17</v>
       </c>
       <c r="E5">
         <v>1</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="G5" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>5</v>
       </c>
       <c r="B6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C6" t="s">
         <v>18</v>
       </c>
-      <c r="C6" t="s">
+      <c r="D6" t="s">
         <v>19</v>
       </c>
-      <c r="D6" t="s">
-        <v>20</v>
-      </c>
       <c r="E6">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="G6" t="s">
-        <v>91</v>
+        <v>79</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -812,22 +753,19 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
+        <v>20</v>
+      </c>
+      <c r="C7" t="s">
         <v>21</v>
       </c>
-      <c r="C7" t="s">
+      <c r="D7" t="s">
         <v>22</v>
-      </c>
-      <c r="D7" t="s">
-        <v>23</v>
       </c>
       <c r="E7">
         <v>0</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="G7" t="s">
-        <v>90</v>
+        <v>66</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -835,22 +773,19 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
+        <v>23</v>
+      </c>
+      <c r="C8" t="s">
         <v>24</v>
       </c>
-      <c r="C8" t="s">
+      <c r="D8" t="s">
         <v>25</v>
       </c>
-      <c r="D8" t="s">
-        <v>26</v>
-      </c>
       <c r="E8">
         <v>2</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="G8" t="s">
-        <v>92</v>
+        <v>67</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -858,22 +793,19 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
+        <v>26</v>
+      </c>
+      <c r="C9" t="s">
         <v>27</v>
       </c>
-      <c r="C9" t="s">
+      <c r="D9" t="s">
         <v>28</v>
       </c>
-      <c r="D9" t="s">
-        <v>29</v>
-      </c>
       <c r="E9">
         <v>2</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="G9" t="s">
-        <v>92</v>
+        <v>68</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -881,45 +813,39 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
+        <v>29</v>
+      </c>
+      <c r="C10" t="s">
+        <v>12</v>
+      </c>
+      <c r="D10" t="s">
         <v>30</v>
       </c>
-      <c r="C10" t="s">
-        <v>13</v>
-      </c>
-      <c r="D10" t="s">
-        <v>31</v>
-      </c>
       <c r="E10">
         <v>2</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="G10" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>10</v>
       </c>
       <c r="B11" t="s">
+        <v>31</v>
+      </c>
+      <c r="C11" t="s">
+        <v>9</v>
+      </c>
+      <c r="D11" t="s">
         <v>32</v>
       </c>
-      <c r="C11" t="s">
-        <v>10</v>
-      </c>
-      <c r="D11" t="s">
-        <v>33</v>
-      </c>
       <c r="E11">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="G11" t="s">
-        <v>93</v>
+        <v>81</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.3">
@@ -927,22 +853,19 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C12" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D12" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="E12">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="G12" t="s">
-        <v>94</v>
+        <v>82</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.3">
@@ -950,22 +873,19 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="C13" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D13" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="E13">
         <v>2</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="G13" t="s">
-        <v>95</v>
+        <v>70</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.3">
@@ -973,22 +893,19 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C14" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D14" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="E14">
         <v>2</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="G14" t="s">
-        <v>92</v>
+        <v>71</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.3">
@@ -996,22 +913,19 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
+        <v>39</v>
+      </c>
+      <c r="C15" t="s">
+        <v>40</v>
+      </c>
+      <c r="D15" t="s">
         <v>41</v>
       </c>
-      <c r="C15" t="s">
-        <v>42</v>
-      </c>
-      <c r="D15" t="s">
-        <v>43</v>
-      </c>
       <c r="E15">
         <v>2</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="G15" t="s">
-        <v>96</v>
+        <v>83</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.3">
@@ -1019,191 +933,164 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="C16" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="D16" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="E16">
         <v>2</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="G16" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>16</v>
       </c>
       <c r="B17" t="s">
+        <v>44</v>
+      </c>
+      <c r="C17" t="s">
+        <v>45</v>
+      </c>
+      <c r="D17" t="s">
         <v>46</v>
       </c>
-      <c r="C17" t="s">
-        <v>47</v>
-      </c>
-      <c r="D17" t="s">
-        <v>48</v>
-      </c>
       <c r="E17">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="G17" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="C18" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="D18" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="E18">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="G18" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="C19" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D19" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="E19">
         <v>2</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="G19" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>19</v>
       </c>
       <c r="B20" t="s">
+        <v>52</v>
+      </c>
+      <c r="C20" t="s">
+        <v>53</v>
+      </c>
+      <c r="D20" t="s">
+        <v>54</v>
+      </c>
+      <c r="E20">
+        <v>2</v>
+      </c>
+      <c r="F20" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="C20" t="s">
-        <v>56</v>
-      </c>
-      <c r="D20" t="s">
-        <v>57</v>
-      </c>
-      <c r="E20">
-        <v>2</v>
-      </c>
-      <c r="F20" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="G20" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>20</v>
       </c>
       <c r="B21" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="C21" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="D21" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="E21">
         <v>2</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="G21" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="22" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>21</v>
       </c>
       <c r="B22" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="C22" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="D22" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="E22">
         <v>1</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="G22" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>22</v>
       </c>
       <c r="B23" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="C23" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="D23" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="E23">
         <v>2</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="G23" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="E24">
-        <v>31</v>
-      </c>
-      <c r="G24">
-        <v>38.5</v>
+        <v>76</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E24" t="s">
+        <v>86</v>
       </c>
     </row>
   </sheetData>

</xml_diff>